<commit_message>
fix(hrm): EXP-75 close re-review blockers #1-#7/#9/#2
Auth onboarding download, fileId claim + dedicated VO, onboarding-only
attachment limits, 20MB upload config, sparse three-state roster update,
migration soft-delete dedupe, and synthetic TEST_* fixtures/evidence.
</commit_message>
<xml_diff>
--- a/docs/superpowers/verification/exp75-evidence/文枢花名册-evidence.xlsx
+++ b/docs/superpowers/verification/exp75-evidence/文枢花名册-evidence.xlsx
@@ -375,7 +375,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>钟伟</t>
+          <t>TEST_EMP_NAME</t>
         </is>
       </c>
       <c r="H2" s="2"/>
@@ -385,12 +385,12 @@
       <c r="L2" s="2"/>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>430981198311201111</t>
+          <t>TEST_ID_CARD_000000000000</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>15995408684</t>
+          <t>10000000000</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -430,7 +430,7 @@
       <c r="AO2" s="2"/>
       <c r="AP2" s="2" t="inlineStr">
         <is>
-          <t>6217231102004496773</t>
+          <t>TEST_BANK_ACCT_0000</t>
         </is>
       </c>
       <c r="AQ2" s="2"/>

</xml_diff>